<commit_message>
Update notebooks and docs with corrected MA Vuln metrics
- Re-execute rq2_vulnerability_detection_analysis notebook with corrected
  classification reports (regenerated by reeval script)
- Update ANALYSIS_SUMMARY_RQ2.md with corrected metrics:
  - MA F1: 36.37% → 43.56%
  - DA F1: 44.22% → 44.91%
  - DA vs MA gap narrowed from ~8% to ~1.4%
- Regenerate analysis visualizations and Excel export

Key insight: The narrowed gap confirms both DA and MA hover around
~45% F1 (random level for balanced dataset), validating that multi-agent
approaches don't improve vulnerability detection accuracy.
</commit_message>
<xml_diff>
--- a/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
+++ b/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
@@ -8,6 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DA vs MA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompting Strategy" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Size" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Type" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy Analysis" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +511,17 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>efficiency_f1_per_kwh</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>avg_output_tokens</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>config</t>
         </is>
       </c>
     </row>
@@ -537,30 +552,30 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.4940593449889189</v>
+        <v>0.25</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4781433077963046</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I2" t="n">
         <v>386</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235757_classification_report.csv</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>49.40593449889189</v>
+        <v>25</v>
       </c>
       <c r="L2" t="n">
-        <v>49.48186528497409</v>
+        <v>50</v>
       </c>
       <c r="M2" t="n">
-        <v>47.81433077963046</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="N2" t="n">
         <v>0.2769755148910969</v>
@@ -569,7 +584,15 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P2" t="n">
-        <v>246.1917098445596</v>
+        <v>120.3475814331081</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>53</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -580,7 +603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -599,45 +622,53 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.247402615017361</v>
+        <v>0.25</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4973958333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3304438405797101</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I3" t="n">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-005140_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235757_classification_report.csv</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>24.7402615017361</v>
+        <v>25</v>
       </c>
       <c r="L3" t="n">
-        <v>49.73958333333333</v>
+        <v>50</v>
       </c>
       <c r="M3" t="n">
-        <v>33.04438405797101</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="N3" t="n">
-        <v>1.066736043243749</v>
+        <v>0.2769755148910969</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1813909970012966</v>
+        <v>0.04709774747862676</v>
       </c>
       <c r="P3" t="n">
-        <v>2606.9453125</v>
+        <v>120.3475814331081</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>246.1917098445596</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pod2</t>
+          <t>pod1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,7 +683,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -661,50 +692,58 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.4803715506136009</v>
+        <v>0.4940593449889189</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4922279792746113</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H4" t="n">
-        <v>0.401909941816342</v>
+        <v>0.4781433077963046</v>
       </c>
       <c r="I4" t="n">
         <v>386</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_classification_report.csv</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>48.03715506136009</v>
+        <v>49.40593449889189</v>
       </c>
       <c r="L4" t="n">
-        <v>49.22279792746113</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M4" t="n">
-        <v>40.1909941816342</v>
+        <v>47.81433077963046</v>
       </c>
       <c r="N4" t="n">
-        <v>2.149316081830814</v>
+        <v>0.2769755148910969</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3654761545027571</v>
+        <v>0.04709774747862676</v>
       </c>
       <c r="P4" t="n">
-        <v>1447.80829015544</v>
+        <v>172.6301720151343</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>53</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pod2</t>
+          <t>pod1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -714,7 +753,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -723,50 +762,58 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.24543416447944</v>
+        <v>0.4940593449889189</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4895833333333333</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3269594988344988</v>
+        <v>0.4781433077963046</v>
       </c>
       <c r="I5" t="n">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_classification_report.csv</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>24.543416447944</v>
+        <v>49.40593449889189</v>
       </c>
       <c r="L5" t="n">
-        <v>48.95833333333333</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M5" t="n">
-        <v>32.69594988344988</v>
+        <v>47.81433077963046</v>
       </c>
       <c r="N5" t="n">
-        <v>3.521474491263214</v>
+        <v>0.2769755148910969</v>
       </c>
       <c r="O5" t="n">
-        <v>0.5988020869178703</v>
+        <v>0.04709774747862676</v>
       </c>
       <c r="P5" t="n">
-        <v>10499.75</v>
+        <v>172.6301720151343</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>246.1917098445596</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pod3</t>
+          <t>pod1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -781,54 +828,62 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.4946626106194691</v>
+        <v>0.5099629296081429</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.4973684210526315</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4910991366196326</v>
+        <v>0.3741727571239038</v>
       </c>
       <c r="I6" t="n">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-005140_classification_report.csv</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>49.46626106194691</v>
+        <v>50.99629296081429</v>
       </c>
       <c r="L6" t="n">
-        <v>49.48186528497409</v>
+        <v>49.73684210526315</v>
       </c>
       <c r="M6" t="n">
-        <v>49.10991366196326</v>
+        <v>37.41727571239038</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2265236020906039</v>
+        <v>1.066736043243749</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0385187528702925</v>
+        <v>0.1813909970012966</v>
       </c>
       <c r="P6" t="n">
-        <v>350.5569948186529</v>
+        <v>35.07641459138409</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>2606.9453125</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pod3</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -838,59 +893,67 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.5</v>
+        <v>0.4803715506136009</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5</v>
+        <v>0.4922279792746113</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4124531724437084</v>
+        <v>0.401909941816342</v>
       </c>
       <c r="I7" t="n">
         <v>386</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_classification_report.csv</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>50</v>
+        <v>48.03715506136009</v>
       </c>
       <c r="L7" t="n">
-        <v>50</v>
+        <v>49.22279792746113</v>
       </c>
       <c r="M7" t="n">
-        <v>41.24531724437084</v>
+        <v>40.1909941816342</v>
       </c>
       <c r="N7" t="n">
-        <v>0.3521505092753471</v>
+        <v>2.149316081830814</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0598807290487078</v>
+        <v>0.3654761545027571</v>
       </c>
       <c r="P7" t="n">
-        <v>1294.29274611399</v>
+        <v>18.6994339833902</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1447.80829015544</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pod4</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -905,54 +968,62 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.5284520884520885</v>
+        <v>0.4672924517528835</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5233160621761658</v>
+        <v>0.4708994708994709</v>
       </c>
       <c r="H8" t="n">
-        <v>0.500787224471435</v>
+        <v>0.4400019494492805</v>
       </c>
       <c r="I8" t="n">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_classification_report.csv</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>52.84520884520884</v>
+        <v>46.72924517528835</v>
       </c>
       <c r="L8" t="n">
-        <v>52.33160621761657</v>
+        <v>47.08994708994709</v>
       </c>
       <c r="M8" t="n">
-        <v>50.0787224471435</v>
+        <v>44.00019494492805</v>
       </c>
       <c r="N8" t="n">
-        <v>1.727872051523862</v>
+        <v>3.521474491263214</v>
       </c>
       <c r="O8" t="n">
-        <v>0.2938125472572721</v>
+        <v>0.5988020869178703</v>
       </c>
       <c r="P8" t="n">
-        <v>1156.20725388601</v>
+        <v>12.49482143178735</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>10499.75</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pod4</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -962,7 +1033,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -971,55 +1042,63 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.4993489539181445</v>
+        <v>0.4946626106194691</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4987012987012987</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3364526488004749</v>
+        <v>0.4910991366196326</v>
       </c>
       <c r="I9" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_classification_report.csv</t>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_classification_report.csv</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>49.93489539181445</v>
+        <v>49.46626106194691</v>
       </c>
       <c r="L9" t="n">
-        <v>49.87012987012987</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M9" t="n">
-        <v>33.64526488004748</v>
+        <v>49.10991366196326</v>
       </c>
       <c r="N9" t="n">
-        <v>3.052417913635256</v>
+        <v>0.2265236020906039</v>
       </c>
       <c r="O9" t="n">
-        <v>0.5190422992882794</v>
+        <v>0.0385187528702925</v>
       </c>
       <c r="P9" t="n">
-        <v>9445.148051948052</v>
+        <v>216.7982197383587</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>350.5569948186529</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Few-shot</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>pod5</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1029,121 +1108,137 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.4763480392156863</v>
+        <v>0.4962282587453587</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4844559585492228</v>
+        <v>0.4974093264248704</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4361323379359452</v>
+        <v>0.4547228613870037</v>
       </c>
       <c r="I10" t="n">
         <v>386</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_classification_report.csv</t>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_classification_report.csv</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>47.63480392156863</v>
+        <v>49.62282587453587</v>
       </c>
       <c r="L10" t="n">
-        <v>48.44559585492228</v>
+        <v>49.74093264248704</v>
       </c>
       <c r="M10" t="n">
-        <v>43.61323379359452</v>
+        <v>45.47228613870037</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3170479884975216</v>
+        <v>0.3521505092753471</v>
       </c>
       <c r="O10" t="n">
-        <v>0.053911791108084</v>
+        <v>0.0598807290487078</v>
       </c>
       <c r="P10" t="n">
-        <v>205.9844559585492</v>
+        <v>129.1274183651556</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1294.29274611399</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>4B-Instruct-Few-shot</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pod5</t>
+          <t>pod4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.25</v>
+        <v>0.5284520884520885</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5</v>
+        <v>0.5233160621761658</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.500787224471435</v>
       </c>
       <c r="I11" t="n">
         <v>386</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_classification_report.csv</t>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_classification_report.csv</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>25</v>
+        <v>52.84520884520884</v>
       </c>
       <c r="L11" t="n">
-        <v>50</v>
+        <v>52.33160621761657</v>
       </c>
       <c r="M11" t="n">
-        <v>33.33333333333333</v>
+        <v>50.0787224471435</v>
       </c>
       <c r="N11" t="n">
-        <v>0.6646637712305367</v>
+        <v>1.727872051523862</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1130214216513541</v>
+        <v>0.2938125472572721</v>
       </c>
       <c r="P11" t="n">
-        <v>2314.30829015544</v>
+        <v>28.98288817333295</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1156.20725388601</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pod6</t>
+          <t>pod4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1153,54 +1248,62 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.5353479853479853</v>
+        <v>0.5346423353522745</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5310880829015544</v>
+        <v>0.5225464190981433</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5165216909907479</v>
+        <v>0.4861117547795792</v>
       </c>
       <c r="I12" t="n">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_classification_report.csv</t>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_classification_report.csv</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>53.53479853479853</v>
+        <v>53.46423353522744</v>
       </c>
       <c r="L12" t="n">
-        <v>53.10880829015544</v>
+        <v>52.25464190981432</v>
       </c>
       <c r="M12" t="n">
-        <v>51.65216909907478</v>
+        <v>48.61117547795792</v>
       </c>
       <c r="N12" t="n">
-        <v>1.890200869433597</v>
+        <v>3.052417913635256</v>
       </c>
       <c r="O12" t="n">
-        <v>0.321415426441097</v>
+        <v>0.5190422992882794</v>
       </c>
       <c r="P12" t="n">
-        <v>1288.764248704663</v>
+        <v>15.9254652715836</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>9445.148051948052</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>pod6</t>
+          <t>pod5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1210,7 +1313,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1219,50 +1322,58 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.7506493506493507</v>
+        <v>0.4763480392156863</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5012987012987012</v>
+        <v>0.4844559585492228</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3376355603159727</v>
+        <v>0.4361323379359452</v>
       </c>
       <c r="I13" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_classification_report.csv</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>75.06493506493507</v>
+        <v>47.63480392156863</v>
       </c>
       <c r="L13" t="n">
-        <v>50.12987012987013</v>
+        <v>48.44559585492228</v>
       </c>
       <c r="M13" t="n">
-        <v>33.76355603159727</v>
+        <v>43.61323379359452</v>
       </c>
       <c r="N13" t="n">
-        <v>2.829785599841551</v>
+        <v>0.3170479884975216</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4811852327538565</v>
+        <v>0.053911791108084</v>
       </c>
       <c r="P13" t="n">
-        <v>9235.044155844156</v>
+        <v>137.5603548228645</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>205.9844559585492</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>pod7</t>
+          <t>pod5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1277,54 +1388,62 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.5313265456691751</v>
+        <v>0.4177960195152172</v>
       </c>
       <c r="G14" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.4715025906735751</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5176060206548011</v>
+        <v>0.3683298572116156</v>
       </c>
       <c r="I14" t="n">
         <v>386</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_classification_report.csv</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>53.13265456691752</v>
+        <v>41.77960195152172</v>
       </c>
       <c r="L14" t="n">
-        <v>52.84974093264248</v>
+        <v>47.15025906735751</v>
       </c>
       <c r="M14" t="n">
-        <v>51.76060206548011</v>
+        <v>36.83298572116156</v>
       </c>
       <c r="N14" t="n">
-        <v>0.5986731427653721</v>
+        <v>0.6646637712305367</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1018001772152521</v>
+        <v>0.1130214216513541</v>
       </c>
       <c r="P14" t="n">
-        <v>479.5466321243524</v>
+        <v>55.41596716332257</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>2314.30829015544</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>pod7</t>
+          <t>pod6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1334,59 +1453,67 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.5378660863981736</v>
+        <v>0.5353479853479853</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.5310880829015544</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4974102160537988</v>
+        <v>0.5165216909907479</v>
       </c>
       <c r="I15" t="n">
         <v>386</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_classification_report.csv</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>53.78660863981736</v>
+        <v>53.53479853479853</v>
       </c>
       <c r="L15" t="n">
-        <v>52.84974093264248</v>
+        <v>53.10880829015544</v>
       </c>
       <c r="M15" t="n">
-        <v>49.74102160537988</v>
+        <v>51.65216909907478</v>
       </c>
       <c r="N15" t="n">
-        <v>0.3836358502976715</v>
+        <v>1.890200869433597</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0652345908921669</v>
+        <v>0.321415426441097</v>
       </c>
       <c r="P15" t="n">
-        <v>1438.044041450777</v>
+        <v>27.32628575848263</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1288.764248704663</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>pod8</t>
+          <t>pod6</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1401,105 +1528,660 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.4671860026585056</v>
+        <v>0.5</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4715025906735751</v>
+        <v>0.5</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4535309793471019</v>
+        <v>0.4674102269038978</v>
       </c>
       <c r="I16" t="n">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_classification_report.csv</t>
         </is>
       </c>
       <c r="K16" t="n">
-        <v>46.71860026585055</v>
+        <v>50</v>
       </c>
       <c r="L16" t="n">
-        <v>47.15025906735751</v>
+        <v>50</v>
       </c>
       <c r="M16" t="n">
-        <v>45.35309793471019</v>
+        <v>46.74102269038978</v>
       </c>
       <c r="N16" t="n">
-        <v>1.494887650667461</v>
+        <v>2.82978559984155</v>
       </c>
       <c r="O16" t="n">
-        <v>0.254195180782447</v>
+        <v>0.4811852327538566</v>
       </c>
       <c r="P16" t="n">
-        <v>1226.841968911917</v>
+        <v>16.51751379786757</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>9235.044155844156</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.5313265456691751</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.5176060206548011</v>
+      </c>
+      <c r="I17" t="n">
+        <v>386</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>53.13265456691752</v>
+      </c>
+      <c r="L17" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M17" t="n">
+        <v>51.76060206548011</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.5986731427653721</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.1018001772152521</v>
+      </c>
+      <c r="P17" t="n">
+        <v>86.45886773271499</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>479.5466321243524</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.4779408403053993</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.4870466321243523</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.4280197575213291</v>
+      </c>
+      <c r="I18" t="n">
+        <v>386</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>47.79408403053993</v>
+      </c>
+      <c r="L18" t="n">
+        <v>48.70466321243523</v>
+      </c>
+      <c r="M18" t="n">
+        <v>42.80197575213291</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.3836358502976715</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.0652345908921669</v>
+      </c>
+      <c r="P18" t="n">
+        <v>111.5692803968188</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1438.044041450777</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>pod8</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.4671860026585056</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.4715025906735751</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.4535309793471019</v>
+      </c>
+      <c r="I19" t="n">
+        <v>386</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>46.71860026585055</v>
+      </c>
+      <c r="L19" t="n">
+        <v>47.15025906735751</v>
+      </c>
+      <c r="M19" t="n">
+        <v>45.35309793471019</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1.494887650667461</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.254195180782447</v>
+      </c>
+      <c r="P19" t="n">
+        <v>30.33880032018475</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1226.841968911917</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Multi-Agent</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>30B</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Thinking</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>0.4986979166666667</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.4973958333333333</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.3350160256410256</v>
-      </c>
-      <c r="I17" t="n">
-        <v>384</v>
-      </c>
-      <c r="J17" t="inlineStr">
+      <c r="F20" t="n">
+        <v>0.5115785174596692</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.5079365079365079</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.4659394749635391</v>
+      </c>
+      <c r="I20" t="n">
+        <v>378</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-090122_classification_report.csv</t>
         </is>
       </c>
-      <c r="K17" t="n">
-        <v>49.86979166666667</v>
-      </c>
-      <c r="L17" t="n">
-        <v>49.73958333333333</v>
-      </c>
-      <c r="M17" t="n">
-        <v>33.50160256410256</v>
-      </c>
-      <c r="N17" t="n">
-        <v>2.61932938577809</v>
-      </c>
-      <c r="O17" t="n">
+      <c r="K20" t="n">
+        <v>51.15785174596692</v>
+      </c>
+      <c r="L20" t="n">
+        <v>50.79365079365079</v>
+      </c>
+      <c r="M20" t="n">
+        <v>46.59394749635391</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.619329385778091</v>
+      </c>
+      <c r="O20" t="n">
         <v>0.4453986267458636</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P20" t="n">
+        <v>17.78850256456495</v>
+      </c>
+      <c r="Q20" t="n">
         <v>8683.247395833334</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>agent_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>precision_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>recall_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>f1_score_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>47.30837963961589</v>
+      </c>
+      <c r="C2" t="n">
+        <v>50.23028209556706</v>
+      </c>
+      <c r="D2" t="n">
+        <v>45.87848858850715</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>48.94301690923682</v>
+      </c>
+      <c r="C3" t="n">
+        <v>49.43386710261939</v>
+      </c>
+      <c r="D3" t="n">
+        <v>43.55885799175186</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>prompting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>precision_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>recall_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>f1_score_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>50.52521499077424</v>
+      </c>
+      <c r="C2" t="n">
+        <v>50.41342000762226</v>
+      </c>
+      <c r="D2" t="n">
+        <v>47.47271512180527</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>45.90198134491595</v>
+      </c>
+      <c r="C3" t="n">
+        <v>49.35956840223119</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42.39950447290411</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model_size</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>precision_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>recall_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>f1_score_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>48.96904937714547</v>
+      </c>
+      <c r="C2" t="n">
+        <v>49.77537215231516</v>
+      </c>
+      <c r="D2" t="n">
+        <v>45.66862931911222</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>47.28523966814152</v>
+      </c>
+      <c r="C3" t="n">
+        <v>49.92672205139306</v>
+      </c>
+      <c r="D3" t="n">
+        <v>44.00313629752016</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>precision_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>recall_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>f1_score_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>46.09249542963742</v>
+      </c>
+      <c r="C2" t="n">
+        <v>49.51019604278398</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.12843743982077</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>50.31088664546259</v>
+      </c>
+      <c r="C3" t="n">
+        <v>50.24396391200035</v>
+      </c>
+      <c r="D3" t="n">
+        <v>46.65266553402404</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>agent_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>energy_kwh</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>emissions_kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.9953858240657139</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1692583916816061</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.811274195570677</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.3079944980374244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(analysis): Regenerate all notebooks and plots after vuln think-tag parsing fix
Re-run 7 analysis notebooks to reflect corrected vulnerability metrics
from commit 688957a. Regenerated vuln_detection_master_dataset.csv,
updated 2 executed notebook copies, and added Data Quality Note #6
documenting the think-tag parsing bug resolution in results/README.md.
</commit_message>
<xml_diff>
--- a/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
+++ b/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,30 +552,30 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.25</v>
+        <v>0.4940593449889189</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4781433077963046</v>
       </c>
       <c r="I2" t="n">
         <v>386</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235757_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>25</v>
+        <v>49.40593449889189</v>
       </c>
       <c r="L2" t="n">
-        <v>50</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M2" t="n">
-        <v>33.33333333333333</v>
+        <v>47.81433077963046</v>
       </c>
       <c r="N2" t="n">
         <v>0.2769755148910969</v>
@@ -584,10 +584,10 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P2" t="n">
-        <v>120.3475814331081</v>
+        <v>172.6301720151343</v>
       </c>
       <c r="Q2" t="n">
-        <v>53</v>
+        <v>246.1917098445596</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -622,30 +622,30 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.25</v>
+        <v>0.4940593449889189</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4781433077963046</v>
       </c>
       <c r="I3" t="n">
         <v>386</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235757_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>25</v>
+        <v>49.40593449889189</v>
       </c>
       <c r="L3" t="n">
-        <v>50</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M3" t="n">
-        <v>33.33333333333333</v>
+        <v>47.81433077963046</v>
       </c>
       <c r="N3" t="n">
         <v>0.2769755148910969</v>
@@ -654,7 +654,7 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P3" t="n">
-        <v>120.3475814331081</v>
+        <v>172.6301720151343</v>
       </c>
       <c r="Q3" t="n">
         <v>246.1917098445596</v>
@@ -727,7 +727,7 @@
         <v>172.6301720151343</v>
       </c>
       <c r="Q4" t="n">
-        <v>53</v>
+        <v>246.1917098445596</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -762,42 +762,42 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.4940593449889189</v>
+        <v>0.2526109483506944</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5026041666666666</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4781433077963046</v>
+        <v>0.3362308636626228</v>
       </c>
       <c r="I5" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251115-235404_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-005140_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>49.40593449889189</v>
+        <v>25.26109483506944</v>
       </c>
       <c r="L5" t="n">
-        <v>49.48186528497409</v>
+        <v>50.26041666666666</v>
       </c>
       <c r="M5" t="n">
-        <v>47.81433077963046</v>
+        <v>33.62308636626228</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2769755148910969</v>
+        <v>1.066736043243749</v>
       </c>
       <c r="O5" t="n">
-        <v>0.04709774747862676</v>
+        <v>0.1813909970012966</v>
       </c>
       <c r="P5" t="n">
-        <v>172.6301720151343</v>
+        <v>31.51959341696247</v>
       </c>
       <c r="Q5" t="n">
-        <v>246.1917098445596</v>
+        <v>2606.9453125</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -832,16 +832,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.5099629296081429</v>
+        <v>0.2526109483506944</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4973684210526315</v>
+        <v>0.5026041666666666</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3741727571239038</v>
+        <v>0.3362308636626228</v>
       </c>
       <c r="I6" t="n">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -849,13 +849,13 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>50.99629296081429</v>
+        <v>25.26109483506944</v>
       </c>
       <c r="L6" t="n">
-        <v>49.73684210526315</v>
+        <v>50.26041666666666</v>
       </c>
       <c r="M6" t="n">
-        <v>37.41727571239038</v>
+        <v>33.62308636626228</v>
       </c>
       <c r="N6" t="n">
         <v>1.066736043243749</v>
@@ -864,7 +864,7 @@
         <v>0.1813909970012966</v>
       </c>
       <c r="P6" t="n">
-        <v>35.07641459138409</v>
+        <v>31.51959341696247</v>
       </c>
       <c r="Q6" t="n">
         <v>2606.9453125</v>
@@ -878,12 +878,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pod2</t>
+          <t>pod1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -902,46 +902,46 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.4803715506136009</v>
+        <v>0.6269942434210526</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4922279792746113</v>
+        <v>0.5078125</v>
       </c>
       <c r="H7" t="n">
-        <v>0.401909941816342</v>
+        <v>0.3521282219089811</v>
       </c>
       <c r="I7" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-005140_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>48.03715506136009</v>
+        <v>62.69942434210526</v>
       </c>
       <c r="L7" t="n">
-        <v>49.22279792746113</v>
+        <v>50.78125</v>
       </c>
       <c r="M7" t="n">
-        <v>40.1909941816342</v>
+        <v>35.21282219089811</v>
       </c>
       <c r="N7" t="n">
-        <v>2.149316081830814</v>
+        <v>1.066736043243749</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3654761545027571</v>
+        <v>0.1813909970012966</v>
       </c>
       <c r="P7" t="n">
-        <v>18.6994339833902</v>
+        <v>33.00987382391463</v>
       </c>
       <c r="Q7" t="n">
-        <v>1447.80829015544</v>
+        <v>2606.9453125</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>4B-Thinking-Zero-shot</t>
+          <t>4B-Instruct-Zero-shot</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -972,42 +972,42 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.4672924517528835</v>
+        <v>0.5044118319389201</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4708994708994709</v>
+        <v>0.5025906735751295</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4400019494492805</v>
+        <v>0.445352492141895</v>
       </c>
       <c r="I8" t="n">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>46.72924517528835</v>
+        <v>50.44118319389202</v>
       </c>
       <c r="L8" t="n">
-        <v>47.08994708994709</v>
+        <v>50.25906735751295</v>
       </c>
       <c r="M8" t="n">
-        <v>44.00019494492805</v>
+        <v>44.5352492141895</v>
       </c>
       <c r="N8" t="n">
-        <v>3.521474491263214</v>
+        <v>2.149316081830814</v>
       </c>
       <c r="O8" t="n">
-        <v>0.5988020869178703</v>
+        <v>0.3654761545027571</v>
       </c>
       <c r="P8" t="n">
-        <v>12.49482143178735</v>
+        <v>20.72066067465229</v>
       </c>
       <c r="Q8" t="n">
-        <v>10499.75</v>
+        <v>1447.80829015544</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pod3</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1033,67 +1033,67 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.4946626106194691</v>
+        <v>0.5044118319389201</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5025906735751295</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4910991366196326</v>
+        <v>0.445352492141895</v>
       </c>
       <c r="I9" t="n">
         <v>386</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_classification_report.csv</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>49.46626106194691</v>
+        <v>50.44118319389202</v>
       </c>
       <c r="L9" t="n">
-        <v>49.48186528497409</v>
+        <v>50.25906735751295</v>
       </c>
       <c r="M9" t="n">
-        <v>49.10991366196326</v>
+        <v>44.5352492141895</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2265236020906039</v>
+        <v>2.149316081830814</v>
       </c>
       <c r="O9" t="n">
-        <v>0.0385187528702925</v>
+        <v>0.3654761545027571</v>
       </c>
       <c r="P9" t="n">
-        <v>216.7982197383587</v>
+        <v>20.72066067465229</v>
       </c>
       <c r="Q9" t="n">
-        <v>350.5569948186529</v>
+        <v>1447.80829015544</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>4B-Instruct-Few-shot</t>
+          <t>4B-Thinking-Zero-shot</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>pod3</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1103,67 +1103,67 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.4962282587453587</v>
+        <v>0.5044118319389201</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4974093264248704</v>
+        <v>0.5025906735751295</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4547228613870037</v>
+        <v>0.445352492141895</v>
       </c>
       <c r="I10" t="n">
         <v>386</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_classification_report.csv</t>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-000135_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>49.62282587453587</v>
+        <v>50.44118319389202</v>
       </c>
       <c r="L10" t="n">
-        <v>49.74093264248704</v>
+        <v>50.25906735751295</v>
       </c>
       <c r="M10" t="n">
-        <v>45.47228613870037</v>
+        <v>44.5352492141895</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3521505092753471</v>
+        <v>2.149316081830814</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0598807290487078</v>
+        <v>0.3654761545027571</v>
       </c>
       <c r="P10" t="n">
-        <v>129.1274183651556</v>
+        <v>20.72066067465229</v>
       </c>
       <c r="Q10" t="n">
-        <v>1294.29274611399</v>
+        <v>1447.80829015544</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>4B-Instruct-Few-shot</t>
+          <t>4B-Thinking-Zero-shot</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pod4</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1178,57 +1178,57 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.5284520884520885</v>
+        <v>0.4928319863981629</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5233160621761658</v>
+        <v>0.4947916666666667</v>
       </c>
       <c r="H11" t="n">
-        <v>0.500787224471435</v>
+        <v>0.416238124661077</v>
       </c>
       <c r="I11" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>52.84520884520884</v>
+        <v>49.28319863981629</v>
       </c>
       <c r="L11" t="n">
-        <v>52.33160621761657</v>
+        <v>49.47916666666667</v>
       </c>
       <c r="M11" t="n">
-        <v>50.0787224471435</v>
+        <v>41.6238124661077</v>
       </c>
       <c r="N11" t="n">
-        <v>1.727872051523862</v>
+        <v>3.521474491263214</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2938125472572721</v>
+        <v>0.5988020869178703</v>
       </c>
       <c r="P11" t="n">
-        <v>28.98288817333295</v>
+        <v>11.81999545059221</v>
       </c>
       <c r="Q11" t="n">
-        <v>1156.20725388601</v>
+        <v>10499.75</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>4B-Thinking-Few-shot</t>
+          <t>4B-Thinking-Zero-shot</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pod4</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1248,72 +1248,72 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Few-shot</t>
+          <t>Zero-shot</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.5346423353522745</v>
+        <v>0.4726321489886796</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5225464190981433</v>
+        <v>0.484375</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4861117547795792</v>
+        <v>0.4118132239382239</v>
       </c>
       <c r="I12" t="n">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>53.46423353522744</v>
+        <v>47.26321489886796</v>
       </c>
       <c r="L12" t="n">
-        <v>52.25464190981432</v>
+        <v>48.4375</v>
       </c>
       <c r="M12" t="n">
-        <v>48.61117547795792</v>
+        <v>41.18132239382239</v>
       </c>
       <c r="N12" t="n">
-        <v>3.052417913635256</v>
+        <v>3.521474491263214</v>
       </c>
       <c r="O12" t="n">
-        <v>0.5190422992882794</v>
+        <v>0.5988020869178703</v>
       </c>
       <c r="P12" t="n">
-        <v>15.9254652715836</v>
+        <v>11.69434067916532</v>
       </c>
       <c r="Q12" t="n">
-        <v>9445.148051948052</v>
+        <v>10499.75</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>4B-Thinking-Few-shot</t>
+          <t>4B-Thinking-Zero-shot</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>pod5</t>
+          <t>pod2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Instruct</t>
+          <t>Thinking</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1322,63 +1322,63 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.4763480392156863</v>
+        <v>0.4726321489886796</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4844559585492228</v>
+        <v>0.484375</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4361323379359452</v>
+        <v>0.4118132239382239</v>
       </c>
       <c r="I13" t="n">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_classification_report.csv</t>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-052135_classification_report.csv</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>47.63480392156863</v>
+        <v>47.26321489886796</v>
       </c>
       <c r="L13" t="n">
-        <v>48.44559585492228</v>
+        <v>48.4375</v>
       </c>
       <c r="M13" t="n">
-        <v>43.61323379359452</v>
+        <v>41.18132239382239</v>
       </c>
       <c r="N13" t="n">
-        <v>0.3170479884975216</v>
+        <v>3.521474491263214</v>
       </c>
       <c r="O13" t="n">
-        <v>0.053911791108084</v>
+        <v>0.5988020869178703</v>
       </c>
       <c r="P13" t="n">
-        <v>137.5603548228645</v>
+        <v>11.69434067916532</v>
       </c>
       <c r="Q13" t="n">
-        <v>205.9844559585492</v>
+        <v>10499.75</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>30B-Instruct-Zero-shot</t>
+          <t>4B-Thinking-Zero-shot</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>pod5</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1388,57 +1388,57 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.4177960195152172</v>
+        <v>0.4946626106194691</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4715025906735751</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3683298572116156</v>
+        <v>0.4910991366196326</v>
       </c>
       <c r="I14" t="n">
         <v>386</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_classification_report.csv</t>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>41.77960195152172</v>
+        <v>49.46626106194691</v>
       </c>
       <c r="L14" t="n">
-        <v>47.15025906735751</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M14" t="n">
-        <v>36.83298572116156</v>
+        <v>49.10991366196326</v>
       </c>
       <c r="N14" t="n">
-        <v>0.6646637712305367</v>
+        <v>0.2265236020906039</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1130214216513541</v>
+        <v>0.0385187528702925</v>
       </c>
       <c r="P14" t="n">
-        <v>55.41596716332257</v>
+        <v>216.7982197383587</v>
       </c>
       <c r="Q14" t="n">
-        <v>2314.30829015544</v>
+        <v>350.5569948186529</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>30B-Instruct-Zero-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>pod6</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1448,147 +1448,147 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.5353479853479853</v>
+        <v>0.4946626106194691</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5310880829015544</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H15" t="n">
-        <v>0.5165216909907479</v>
+        <v>0.4910991366196326</v>
       </c>
       <c r="I15" t="n">
         <v>386</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_classification_report.csv</t>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_classification_report.csv</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>53.53479853479853</v>
+        <v>49.46626106194691</v>
       </c>
       <c r="L15" t="n">
-        <v>53.10880829015544</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M15" t="n">
-        <v>51.65216909907478</v>
+        <v>49.10991366196326</v>
       </c>
       <c r="N15" t="n">
-        <v>1.890200869433597</v>
+        <v>0.2265236020906039</v>
       </c>
       <c r="O15" t="n">
-        <v>0.321415426441097</v>
+        <v>0.0385187528702925</v>
       </c>
       <c r="P15" t="n">
-        <v>27.32628575848263</v>
+        <v>216.7982197383587</v>
       </c>
       <c r="Q15" t="n">
-        <v>1288.764248704663</v>
+        <v>350.5569948186529</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>30B-Thinking-Zero-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>pod6</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Dual-Agent</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Zero-shot</t>
+          <t>Few-shot</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.5</v>
+        <v>0.4946626106194691</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5</v>
+        <v>0.4948186528497409</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4674102269038978</v>
+        <v>0.4910991366196326</v>
       </c>
       <c r="I16" t="n">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_classification_report.csv</t>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Instruct-2507_vuln_20251116-002738_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K16" t="n">
-        <v>50</v>
+        <v>49.46626106194691</v>
       </c>
       <c r="L16" t="n">
-        <v>50</v>
+        <v>49.48186528497409</v>
       </c>
       <c r="M16" t="n">
-        <v>46.74102269038978</v>
+        <v>49.10991366196326</v>
       </c>
       <c r="N16" t="n">
-        <v>2.82978559984155</v>
+        <v>0.2265236020906039</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4811852327538566</v>
+        <v>0.0385187528702925</v>
       </c>
       <c r="P16" t="n">
-        <v>16.51751379786757</v>
+        <v>216.7982197383587</v>
       </c>
       <c r="Q16" t="n">
-        <v>9235.044155844156</v>
+        <v>350.5569948186529</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>30B-Thinking-Zero-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>pod7</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1602,53 +1602,53 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.5313265456691751</v>
+        <v>0.5</v>
       </c>
       <c r="G17" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.5</v>
       </c>
       <c r="H17" t="n">
-        <v>0.5176060206548011</v>
+        <v>0.4124531724437084</v>
       </c>
       <c r="I17" t="n">
         <v>386</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_classification_report.csv</t>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_strict_classification_report.csv</t>
         </is>
       </c>
       <c r="K17" t="n">
-        <v>53.13265456691752</v>
+        <v>50</v>
       </c>
       <c r="L17" t="n">
-        <v>52.84974093264248</v>
+        <v>50</v>
       </c>
       <c r="M17" t="n">
-        <v>51.76060206548011</v>
+        <v>41.24531724437084</v>
       </c>
       <c r="N17" t="n">
-        <v>0.5986731427653721</v>
+        <v>0.3521505092753471</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1018001772152521</v>
+        <v>0.0598807290487078</v>
       </c>
       <c r="P17" t="n">
-        <v>86.45886773271499</v>
+        <v>117.124116416146</v>
       </c>
       <c r="Q17" t="n">
-        <v>479.5466321243524</v>
+        <v>1294.29274611399</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>30B-Instruct-Few-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>pod7</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1672,68 +1672,68 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.4779408403053993</v>
+        <v>0.5</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4870466321243523</v>
+        <v>0.5</v>
       </c>
       <c r="H18" t="n">
-        <v>0.4280197575213291</v>
+        <v>0.4124531724437084</v>
       </c>
       <c r="I18" t="n">
         <v>386</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_classification_report.csv</t>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_classification_report.csv</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>47.79408403053993</v>
+        <v>50</v>
       </c>
       <c r="L18" t="n">
-        <v>48.70466321243523</v>
+        <v>50</v>
       </c>
       <c r="M18" t="n">
-        <v>42.80197575213291</v>
+        <v>41.24531724437084</v>
       </c>
       <c r="N18" t="n">
-        <v>0.3836358502976715</v>
+        <v>0.3521505092753471</v>
       </c>
       <c r="O18" t="n">
-        <v>0.0652345908921669</v>
+        <v>0.0598807290487078</v>
       </c>
       <c r="P18" t="n">
-        <v>111.5692803968188</v>
+        <v>117.124116416146</v>
       </c>
       <c r="Q18" t="n">
-        <v>1438.044041450777</v>
+        <v>1294.29274611399</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>30B-Instruct-Few-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pod8</t>
+          <t>pod3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dual-Agent</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>30B</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Thinking</t>
+          <t>Instruct</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1742,114 +1742,2144 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.4671860026585056</v>
+        <v>0.5</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4715025906735751</v>
+        <v>0.5</v>
       </c>
       <c r="H19" t="n">
-        <v>0.4535309793471019</v>
+        <v>0.4124531724437084</v>
       </c>
       <c r="I19" t="n">
         <v>386</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_classification_report.csv</t>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Instruct-2507_20251116-011412_conservative_classification_report.csv</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>46.71860026585055</v>
+        <v>50</v>
       </c>
       <c r="L19" t="n">
-        <v>47.15025906735751</v>
+        <v>50</v>
       </c>
       <c r="M19" t="n">
-        <v>45.35309793471019</v>
+        <v>41.24531724437084</v>
       </c>
       <c r="N19" t="n">
-        <v>1.494887650667461</v>
+        <v>0.3521505092753471</v>
       </c>
       <c r="O19" t="n">
-        <v>0.254195180782447</v>
+        <v>0.0598807290487078</v>
       </c>
       <c r="P19" t="n">
-        <v>30.33880032018475</v>
+        <v>117.124116416146</v>
       </c>
       <c r="Q19" t="n">
-        <v>1226.841968911917</v>
+        <v>1294.29274611399</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>30B-Thinking-Few-shot</t>
+          <t>4B-Instruct-Few-shot</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.5026951543080574</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.5025906735751295</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.49772283669486</v>
+      </c>
+      <c r="I20" t="n">
+        <v>386</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>50.26951543080575</v>
+      </c>
+      <c r="L20" t="n">
+        <v>50.25906735751295</v>
+      </c>
+      <c r="M20" t="n">
+        <v>49.772283669486</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1.727872051523862</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.2938125472572721</v>
+      </c>
+      <c r="P20" t="n">
+        <v>28.80553778596646</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1156.20725388601</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.5026951543080574</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.5025906735751295</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.49772283669486</v>
+      </c>
+      <c r="I21" t="n">
+        <v>386</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>50.26951543080575</v>
+      </c>
+      <c r="L21" t="n">
+        <v>50.25906735751295</v>
+      </c>
+      <c r="M21" t="n">
+        <v>49.772283669486</v>
+      </c>
+      <c r="N21" t="n">
+        <v>1.727872051523862</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.2938125472572721</v>
+      </c>
+      <c r="P21" t="n">
+        <v>28.80553778596646</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1156.20725388601</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.5026951543080574</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.5025906735751295</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.49772283669486</v>
+      </c>
+      <c r="I22" t="n">
+        <v>386</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-4B-Thinking-2507_vuln_20251116-003215_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>50.26951543080575</v>
+      </c>
+      <c r="L22" t="n">
+        <v>50.25906735751295</v>
+      </c>
+      <c r="M22" t="n">
+        <v>49.772283669486</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1.727872051523862</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.2938125472572721</v>
+      </c>
+      <c r="P22" t="n">
+        <v>28.80553778596646</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1156.20725388601</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.5359407385814383</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.535064935064935</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.5328528942135269</v>
+      </c>
+      <c r="I23" t="n">
+        <v>385</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>53.59407385814383</v>
+      </c>
+      <c r="L23" t="n">
+        <v>53.5064935064935</v>
+      </c>
+      <c r="M23" t="n">
+        <v>53.28528942135269</v>
+      </c>
+      <c r="N23" t="n">
+        <v>3.052417913635256</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.5190422992882794</v>
+      </c>
+      <c r="P23" t="n">
+        <v>17.45674770919325</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>9445.148051948052</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.5359407385814383</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.535064935064935</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.5328528942135269</v>
+      </c>
+      <c r="I24" t="n">
+        <v>385</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>53.59407385814383</v>
+      </c>
+      <c r="L24" t="n">
+        <v>53.5064935064935</v>
+      </c>
+      <c r="M24" t="n">
+        <v>53.28528942135269</v>
+      </c>
+      <c r="N24" t="n">
+        <v>3.052417913635256</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.5190422992882794</v>
+      </c>
+      <c r="P24" t="n">
+        <v>17.45674770919325</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>9445.148051948052</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>pod4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.5418591278793142</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.5402597402597402</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.5365397794992067</v>
+      </c>
+      <c r="I25" t="n">
+        <v>385</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-4B-Thinking-2507_20251116-051514_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>54.18591278793142</v>
+      </c>
+      <c r="L25" t="n">
+        <v>54.02597402597402</v>
+      </c>
+      <c r="M25" t="n">
+        <v>53.65397794992067</v>
+      </c>
+      <c r="N25" t="n">
+        <v>3.052417913635256</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.5190422992882794</v>
+      </c>
+      <c r="P25" t="n">
+        <v>17.5775334400465</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>9445.148051948052</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>4B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.4763480392156863</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.4844559585492228</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.4361323379359452</v>
+      </c>
+      <c r="I26" t="n">
+        <v>386</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>47.63480392156863</v>
+      </c>
+      <c r="L26" t="n">
+        <v>48.44559585492228</v>
+      </c>
+      <c r="M26" t="n">
+        <v>43.61323379359452</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.3170479884975216</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.053911791108084</v>
+      </c>
+      <c r="P26" t="n">
+        <v>137.5603548228645</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>205.9844559585492</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.4763480392156863</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.4844559585492228</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.4361323379359452</v>
+      </c>
+      <c r="I27" t="n">
+        <v>386</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>47.63480392156863</v>
+      </c>
+      <c r="L27" t="n">
+        <v>48.44559585492228</v>
+      </c>
+      <c r="M27" t="n">
+        <v>43.61323379359452</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.3170479884975216</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.053911791108084</v>
+      </c>
+      <c r="P27" t="n">
+        <v>137.5603548228645</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>205.9844559585492</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.4763480392156863</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.4844559585492228</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.4361323379359452</v>
+      </c>
+      <c r="I28" t="n">
+        <v>386</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-022428_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>47.63480392156863</v>
+      </c>
+      <c r="L28" t="n">
+        <v>48.44559585492228</v>
+      </c>
+      <c r="M28" t="n">
+        <v>43.61323379359452</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.3170479884975216</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.053911791108084</v>
+      </c>
+      <c r="P28" t="n">
+        <v>137.5603548228645</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>205.9844559585492</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I29" t="n">
+        <v>386</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>25</v>
+      </c>
+      <c r="L29" t="n">
+        <v>50</v>
+      </c>
+      <c r="M29" t="n">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.6646637712305367</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.1130214216513541</v>
+      </c>
+      <c r="P29" t="n">
+        <v>50.15066982155668</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>2314.30829015544</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I30" t="n">
+        <v>386</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>25</v>
+      </c>
+      <c r="L30" t="n">
+        <v>50</v>
+      </c>
+      <c r="M30" t="n">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.6646637712305367</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.1130214216513541</v>
+      </c>
+      <c r="P30" t="n">
+        <v>50.15066982155668</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>2314.30829015544</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>pod5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I31" t="n">
+        <v>386</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-032753_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>25</v>
+      </c>
+      <c r="L31" t="n">
+        <v>50</v>
+      </c>
+      <c r="M31" t="n">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.6646637712305367</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.1130214216513541</v>
+      </c>
+      <c r="P31" t="n">
+        <v>50.15066982155668</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>2314.30829015544</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.4733499033416183</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.4792746113989637</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.448630209998934</v>
+      </c>
+      <c r="I32" t="n">
+        <v>386</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>47.33499033416183</v>
+      </c>
+      <c r="L32" t="n">
+        <v>47.92746113989637</v>
+      </c>
+      <c r="M32" t="n">
+        <v>44.8630209998934</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1.890200869433597</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.321415426441097</v>
+      </c>
+      <c r="P32" t="n">
+        <v>23.73452563977326</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>1288.764248704663</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0.4733499033416183</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.4792746113989637</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.448630209998934</v>
+      </c>
+      <c r="I33" t="n">
+        <v>386</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>47.33499033416183</v>
+      </c>
+      <c r="L33" t="n">
+        <v>47.92746113989637</v>
+      </c>
+      <c r="M33" t="n">
+        <v>44.8630209998934</v>
+      </c>
+      <c r="N33" t="n">
+        <v>1.890200869433597</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.321415426441097</v>
+      </c>
+      <c r="P33" t="n">
+        <v>23.73452563977326</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>1288.764248704663</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0.4733499033416183</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.4792746113989637</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.448630209998934</v>
+      </c>
+      <c r="I34" t="n">
+        <v>386</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-025425_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>47.33499033416183</v>
+      </c>
+      <c r="L34" t="n">
+        <v>47.92746113989637</v>
+      </c>
+      <c r="M34" t="n">
+        <v>44.8630209998934</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1.890200869433597</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.321415426441097</v>
+      </c>
+      <c r="P34" t="n">
+        <v>23.73452563977326</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1288.764248704663</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0.5327096211340584</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.5194805194805194</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.4692392365008354</v>
+      </c>
+      <c r="I35" t="n">
+        <v>385</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>53.27096211340584</v>
+      </c>
+      <c r="L35" t="n">
+        <v>51.94805194805194</v>
+      </c>
+      <c r="M35" t="n">
+        <v>46.92392365008354</v>
+      </c>
+      <c r="N35" t="n">
+        <v>2.82978559984155</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.4811852327538566</v>
+      </c>
+      <c r="P35" t="n">
+        <v>16.58214800892017</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>9235.044155844156</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0.5327096211340584</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.5194805194805194</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.4692392365008354</v>
+      </c>
+      <c r="I36" t="n">
+        <v>385</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>53.27096211340584</v>
+      </c>
+      <c r="L36" t="n">
+        <v>51.94805194805194</v>
+      </c>
+      <c r="M36" t="n">
+        <v>46.92392365008354</v>
+      </c>
+      <c r="N36" t="n">
+        <v>2.82978559984155</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.4811852327538566</v>
+      </c>
+      <c r="P36" t="n">
+        <v>16.58214800892017</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>9235.044155844156</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>pod6</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Zero-shot</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0.5301627009937412</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.5168831168831168</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.46152083175585</v>
+      </c>
+      <c r="I37" t="n">
+        <v>385</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-zero_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-091327_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>53.01627009937412</v>
+      </c>
+      <c r="L37" t="n">
+        <v>51.68831168831169</v>
+      </c>
+      <c r="M37" t="n">
+        <v>46.152083175585</v>
+      </c>
+      <c r="N37" t="n">
+        <v>2.82978559984155</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.4811852327538566</v>
+      </c>
+      <c r="P37" t="n">
+        <v>16.30939219500206</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>9235.044155844156</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Zero-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>0.5313265456691751</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.5176060206548011</v>
+      </c>
+      <c r="I38" t="n">
+        <v>386</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>53.13265456691752</v>
+      </c>
+      <c r="L38" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M38" t="n">
+        <v>51.76060206548011</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.5986731427653721</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.1018001772152521</v>
+      </c>
+      <c r="P38" t="n">
+        <v>86.45886773271499</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>479.5466321243524</v>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0.5313265456691751</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.5176060206548011</v>
+      </c>
+      <c r="I39" t="n">
+        <v>386</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>53.13265456691752</v>
+      </c>
+      <c r="L39" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M39" t="n">
+        <v>51.76060206548011</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.5986731427653721</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.1018001772152521</v>
+      </c>
+      <c r="P39" t="n">
+        <v>86.45886773271499</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>479.5466321243524</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>0.5313265456691751</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.5176060206548011</v>
+      </c>
+      <c r="I40" t="n">
+        <v>386</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_vuln_20251116-025708_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>53.13265456691752</v>
+      </c>
+      <c r="L40" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M40" t="n">
+        <v>51.76060206548011</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.5986731427653721</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.1018001772152521</v>
+      </c>
+      <c r="P40" t="n">
+        <v>86.45886773271499</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>479.5466321243524</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0.5378660863981736</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.4974102160537988</v>
+      </c>
+      <c r="I41" t="n">
+        <v>386</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>53.78660863981736</v>
+      </c>
+      <c r="L41" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M41" t="n">
+        <v>49.74102160537988</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.3836358502976715</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.0652345908921669</v>
+      </c>
+      <c r="P41" t="n">
+        <v>129.6568648805494</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>1438.044041450777</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>0.5378660863981736</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.4974102160537988</v>
+      </c>
+      <c r="I42" t="n">
+        <v>386</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>53.78660863981736</v>
+      </c>
+      <c r="L42" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M42" t="n">
+        <v>49.74102160537988</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.3836358502976715</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.0652345908921669</v>
+      </c>
+      <c r="P42" t="n">
+        <v>129.6568648805494</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1438.044041450777</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>pod7</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Instruct</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>0.5378660863981736</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.5284974093264249</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.4974102160537988</v>
+      </c>
+      <c r="I43" t="n">
+        <v>386</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Instruct-2507_20251116-043150_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>53.78660863981736</v>
+      </c>
+      <c r="L43" t="n">
+        <v>52.84974093264248</v>
+      </c>
+      <c r="M43" t="n">
+        <v>49.74102160537988</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.3836358502976715</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.0652345908921669</v>
+      </c>
+      <c r="P43" t="n">
+        <v>129.6568648805494</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1438.044041450777</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>30B-Instruct-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>pod8</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>0.5217049032838507</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.5207253886010362</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.515256423310593</v>
+      </c>
+      <c r="I44" t="n">
+        <v>386</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>52.17049032838506</v>
+      </c>
+      <c r="L44" t="n">
+        <v>52.07253886010362</v>
+      </c>
+      <c r="M44" t="n">
+        <v>51.5256423310593</v>
+      </c>
+      <c r="N44" t="n">
+        <v>1.494887650667461</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.254195180782447</v>
+      </c>
+      <c r="P44" t="n">
+        <v>34.46790286082926</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>1226.841968911917</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>0.5217049032838507</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.5207253886010362</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.515256423310593</v>
+      </c>
+      <c r="I45" t="n">
+        <v>386</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>52.17049032838506</v>
+      </c>
+      <c r="L45" t="n">
+        <v>52.07253886010362</v>
+      </c>
+      <c r="M45" t="n">
+        <v>51.5256423310593</v>
+      </c>
+      <c r="N45" t="n">
+        <v>1.494887650667461</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.254195180782447</v>
+      </c>
+      <c r="P45" t="n">
+        <v>34.46790286082926</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1226.841968911917</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Dual-Agent</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>0.5217049032838507</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.5207253886010362</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.515256423310593</v>
+      </c>
+      <c r="I46" t="n">
+        <v>386</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DA-vuln-two-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_vuln_20251116-032211_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>52.17049032838506</v>
+      </c>
+      <c r="L46" t="n">
+        <v>52.07253886010362</v>
+      </c>
+      <c r="M46" t="n">
+        <v>51.5256423310593</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1.494887650667461</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.254195180782447</v>
+      </c>
+      <c r="P46" t="n">
+        <v>34.46790286082926</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1226.841968911917</v>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Multi-Agent</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>30B</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Thinking</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Few-shot</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>0.5115785174596692</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.5079365079365079</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.4659394749635391</v>
-      </c>
-      <c r="I20" t="n">
-        <v>378</v>
-      </c>
-      <c r="J20" t="inlineStr">
+      <c r="F47" t="n">
+        <v>0.5054607965555828</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.5052083333333334</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.5044556962741636</v>
+      </c>
+      <c r="I47" t="n">
+        <v>384</v>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-090122_classification_report.csv</t>
         </is>
       </c>
-      <c r="K20" t="n">
-        <v>51.15785174596692</v>
-      </c>
-      <c r="L20" t="n">
-        <v>50.79365079365079</v>
-      </c>
-      <c r="M20" t="n">
-        <v>46.59394749635391</v>
-      </c>
-      <c r="N20" t="n">
+      <c r="K47" t="n">
+        <v>50.54607965555829</v>
+      </c>
+      <c r="L47" t="n">
+        <v>50.52083333333334</v>
+      </c>
+      <c r="M47" t="n">
+        <v>50.44556962741636</v>
+      </c>
+      <c r="N47" t="n">
         <v>2.619329385778091</v>
       </c>
-      <c r="O20" t="n">
+      <c r="O47" t="n">
         <v>0.4453986267458636</v>
       </c>
-      <c r="P20" t="n">
-        <v>17.78850256456495</v>
-      </c>
-      <c r="Q20" t="n">
+      <c r="P47" t="n">
+        <v>19.25896372610318</v>
+      </c>
+      <c r="Q47" t="n">
         <v>8683.247395833334</v>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>0.5054607965555828</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.5052083333333334</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.5044556962741636</v>
+      </c>
+      <c r="I48" t="n">
+        <v>384</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-090122_conservative_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>50.54607965555829</v>
+      </c>
+      <c r="L48" t="n">
+        <v>50.52083333333334</v>
+      </c>
+      <c r="M48" t="n">
+        <v>50.44556962741636</v>
+      </c>
+      <c r="N48" t="n">
+        <v>2.619329385778091</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.4453986267458636</v>
+      </c>
+      <c r="P48" t="n">
+        <v>19.25896372610318</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>8683.247395833334</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>30B-Thinking-Few-shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>pod8</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Multi-Agent</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>30B</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Thinking</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Few-shot</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>0.5003020069736156</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.4985039712762485</v>
+      </c>
+      <c r="I49" t="n">
+        <v>384</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>MA-vuln-four-few_shot_Qwen-Qwen3-30B-A3B-Thinking-2507_20251116-090122_strict_classification_report.csv</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>50.03020069736156</v>
+      </c>
+      <c r="L49" t="n">
+        <v>50</v>
+      </c>
+      <c r="M49" t="n">
+        <v>49.85039712762485</v>
+      </c>
+      <c r="N49" t="n">
+        <v>2.619329385778091</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.4453986267458636</v>
+      </c>
+      <c r="P49" t="n">
+        <v>19.03174048987216</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>8683.247395833334</v>
+      </c>
+      <c r="R49" t="inlineStr">
         <is>
           <t>30B-Thinking-Few-shot</t>
         </is>
@@ -1898,13 +3928,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>47.30837963961589</v>
+        <v>49.9819791670712</v>
       </c>
       <c r="C2" t="n">
-        <v>50.23028209556706</v>
+        <v>50.09715025906736</v>
       </c>
       <c r="D2" t="n">
-        <v>45.87848858850715</v>
+        <v>47.87428456441207</v>
       </c>
     </row>
     <row r="3">
@@ -1914,13 +3944,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.94301690923682</v>
+        <v>46.47690346700548</v>
       </c>
       <c r="C3" t="n">
-        <v>49.43386710261939</v>
+        <v>50.99460483699877</v>
       </c>
       <c r="D3" t="n">
-        <v>43.55885799175186</v>
+        <v>43.76543718238596</v>
       </c>
     </row>
   </sheetData>
@@ -1966,13 +3996,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50.52521499077424</v>
+        <v>51.62387544151312</v>
       </c>
       <c r="C2" t="n">
-        <v>50.41342000762226</v>
+        <v>51.44247865871895</v>
       </c>
       <c r="D2" t="n">
-        <v>47.47271512180527</v>
+        <v>49.60126812117924</v>
       </c>
     </row>
     <row r="3">
@@ -1982,13 +4012,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45.90198134491595</v>
+        <v>44.83500719256355</v>
       </c>
       <c r="C3" t="n">
-        <v>49.35956840223119</v>
+        <v>49.6492764373472</v>
       </c>
       <c r="D3" t="n">
-        <v>42.39950447290411</v>
+        <v>42.03845362561879</v>
       </c>
     </row>
   </sheetData>
@@ -2034,13 +4064,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48.96904937714547</v>
+        <v>47.82746657113396</v>
       </c>
       <c r="C2" t="n">
-        <v>49.77537215231516</v>
+        <v>50.79422147548767</v>
       </c>
       <c r="D2" t="n">
-        <v>45.66862931911222</v>
+        <v>46.4688345518513</v>
       </c>
     </row>
     <row r="3">
@@ -2050,13 +4080,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47.28523966814152</v>
+        <v>48.63141606294271</v>
       </c>
       <c r="C3" t="n">
-        <v>49.92672205139306</v>
+        <v>50.29753362057847</v>
       </c>
       <c r="D3" t="n">
-        <v>44.00313629752016</v>
+        <v>45.17088719494672</v>
       </c>
     </row>
   </sheetData>
@@ -2102,13 +4132,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>46.09249542963742</v>
+        <v>45.77085008665296</v>
       </c>
       <c r="C2" t="n">
-        <v>49.51019604278398</v>
+        <v>50.44285450849165</v>
       </c>
       <c r="D2" t="n">
-        <v>43.12843743982077</v>
+        <v>43.846343848945</v>
       </c>
     </row>
     <row r="3">
@@ -2118,13 +4148,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50.31088664546259</v>
+        <v>50.68803254742372</v>
       </c>
       <c r="C3" t="n">
-        <v>50.24396391200035</v>
+        <v>50.64890058757448</v>
       </c>
       <c r="D3" t="n">
-        <v>46.65266553402404</v>
+        <v>47.79337789785303</v>
       </c>
     </row>
   </sheetData>
@@ -2165,10 +4195,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9953858240657139</v>
+        <v>1.085187112712541</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1692583916816061</v>
+        <v>0.1845284722069786</v>
       </c>
     </row>
     <row r="3">
@@ -2181,7 +4211,7 @@
         <v>1.811274195570677</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3079944980374244</v>
+        <v>0.3079944980374245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(analysis): Regenerate figures and analysis after DA keyword fallback fix
Re-ran 4 notebooks to update all figures and analysis outputs reflecting
the corrected DA vulnerability predictions (2,597 predictions changed).
</commit_message>
<xml_diff>
--- a/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
+++ b/results/analysis/rq2/rq2_vulnerability_detection_analysis.xlsx
@@ -552,13 +552,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.4940593449889189</v>
+        <v>0.4332087486157253</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.4740932642487047</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4781433077963046</v>
+        <v>0.3790720710012282</v>
       </c>
       <c r="I2" t="n">
         <v>386</v>
@@ -569,13 +569,13 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>49.40593449889189</v>
+        <v>43.32087486157253</v>
       </c>
       <c r="L2" t="n">
-        <v>49.48186528497409</v>
+        <v>47.40932642487047</v>
       </c>
       <c r="M2" t="n">
-        <v>47.81433077963046</v>
+        <v>37.90720710012282</v>
       </c>
       <c r="N2" t="n">
         <v>0.2769755148910969</v>
@@ -584,7 +584,7 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P2" t="n">
-        <v>172.6301720151343</v>
+        <v>136.8612208015118</v>
       </c>
       <c r="Q2" t="n">
         <v>246.1917098445596</v>
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.4940593449889189</v>
+        <v>0.4332087486157253</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.4740932642487047</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4781433077963046</v>
+        <v>0.3790720710012282</v>
       </c>
       <c r="I3" t="n">
         <v>386</v>
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>49.40593449889189</v>
+        <v>43.32087486157253</v>
       </c>
       <c r="L3" t="n">
-        <v>49.48186528497409</v>
+        <v>47.40932642487047</v>
       </c>
       <c r="M3" t="n">
-        <v>47.81433077963046</v>
+        <v>37.90720710012282</v>
       </c>
       <c r="N3" t="n">
         <v>0.2769755148910969</v>
@@ -654,7 +654,7 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P3" t="n">
-        <v>172.6301720151343</v>
+        <v>136.8612208015118</v>
       </c>
       <c r="Q3" t="n">
         <v>246.1917098445596</v>
@@ -692,13 +692,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.4940593449889189</v>
+        <v>0.4332087486157253</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.4740932642487047</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4781433077963046</v>
+        <v>0.3790720710012282</v>
       </c>
       <c r="I4" t="n">
         <v>386</v>
@@ -709,13 +709,13 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>49.40593449889189</v>
+        <v>43.32087486157253</v>
       </c>
       <c r="L4" t="n">
-        <v>49.48186528497409</v>
+        <v>47.40932642487047</v>
       </c>
       <c r="M4" t="n">
-        <v>47.81433077963046</v>
+        <v>37.90720710012282</v>
       </c>
       <c r="N4" t="n">
         <v>0.2769755148910969</v>
@@ -724,7 +724,7 @@
         <v>0.04709774747862676</v>
       </c>
       <c r="P4" t="n">
-        <v>172.6301720151343</v>
+        <v>136.8612208015118</v>
       </c>
       <c r="Q4" t="n">
         <v>246.1917098445596</v>
@@ -1392,13 +1392,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.4946626106194691</v>
+        <v>0.6128843582887701</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5362694300518135</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4910991366196326</v>
+        <v>0.4415066887604575</v>
       </c>
       <c r="I14" t="n">
         <v>386</v>
@@ -1409,13 +1409,13 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>49.46626106194691</v>
+        <v>61.28843582887701</v>
       </c>
       <c r="L14" t="n">
-        <v>49.48186528497409</v>
+        <v>53.62694300518135</v>
       </c>
       <c r="M14" t="n">
-        <v>49.10991366196326</v>
+        <v>44.15066887604575</v>
       </c>
       <c r="N14" t="n">
         <v>0.2265236020906039</v>
@@ -1424,7 +1424,7 @@
         <v>0.0385187528702925</v>
       </c>
       <c r="P14" t="n">
-        <v>216.7982197383587</v>
+        <v>194.9053805809893</v>
       </c>
       <c r="Q14" t="n">
         <v>350.5569948186529</v>
@@ -1462,13 +1462,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.4946626106194691</v>
+        <v>0.6128843582887701</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5362694300518135</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4910991366196326</v>
+        <v>0.4415066887604575</v>
       </c>
       <c r="I15" t="n">
         <v>386</v>
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>49.46626106194691</v>
+        <v>61.28843582887701</v>
       </c>
       <c r="L15" t="n">
-        <v>49.48186528497409</v>
+        <v>53.62694300518135</v>
       </c>
       <c r="M15" t="n">
-        <v>49.10991366196326</v>
+        <v>44.15066887604575</v>
       </c>
       <c r="N15" t="n">
         <v>0.2265236020906039</v>
@@ -1494,7 +1494,7 @@
         <v>0.0385187528702925</v>
       </c>
       <c r="P15" t="n">
-        <v>216.7982197383587</v>
+        <v>194.9053805809893</v>
       </c>
       <c r="Q15" t="n">
         <v>350.5569948186529</v>
@@ -1532,13 +1532,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.4946626106194691</v>
+        <v>0.6128843582887701</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4948186528497409</v>
+        <v>0.5362694300518135</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4910991366196326</v>
+        <v>0.4415066887604575</v>
       </c>
       <c r="I16" t="n">
         <v>386</v>
@@ -1549,13 +1549,13 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>49.46626106194691</v>
+        <v>61.28843582887701</v>
       </c>
       <c r="L16" t="n">
-        <v>49.48186528497409</v>
+        <v>53.62694300518135</v>
       </c>
       <c r="M16" t="n">
-        <v>49.10991366196326</v>
+        <v>44.15066887604575</v>
       </c>
       <c r="N16" t="n">
         <v>0.2265236020906039</v>
@@ -1564,7 +1564,7 @@
         <v>0.0385187528702925</v>
       </c>
       <c r="P16" t="n">
-        <v>216.7982197383587</v>
+        <v>194.9053805809893</v>
       </c>
       <c r="Q16" t="n">
         <v>350.5569948186529</v>
@@ -2232,13 +2232,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.4763480392156863</v>
+        <v>0.5</v>
       </c>
       <c r="G26" t="n">
-        <v>0.4844559585492228</v>
+        <v>0.5</v>
       </c>
       <c r="H26" t="n">
-        <v>0.4361323379359452</v>
+        <v>0.3978256476579234</v>
       </c>
       <c r="I26" t="n">
         <v>386</v>
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>47.63480392156863</v>
+        <v>50</v>
       </c>
       <c r="L26" t="n">
-        <v>48.44559585492228</v>
+        <v>50</v>
       </c>
       <c r="M26" t="n">
-        <v>43.61323379359452</v>
+        <v>39.78256476579234</v>
       </c>
       <c r="N26" t="n">
         <v>0.3170479884975216</v>
@@ -2264,7 +2264,7 @@
         <v>0.053911791108084</v>
       </c>
       <c r="P26" t="n">
-        <v>137.5603548228645</v>
+        <v>125.4780544557952</v>
       </c>
       <c r="Q26" t="n">
         <v>205.9844559585492</v>
@@ -2302,13 +2302,13 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.4763480392156863</v>
+        <v>0.5</v>
       </c>
       <c r="G27" t="n">
-        <v>0.4844559585492228</v>
+        <v>0.5</v>
       </c>
       <c r="H27" t="n">
-        <v>0.4361323379359452</v>
+        <v>0.3978256476579234</v>
       </c>
       <c r="I27" t="n">
         <v>386</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>47.63480392156863</v>
+        <v>50</v>
       </c>
       <c r="L27" t="n">
-        <v>48.44559585492228</v>
+        <v>50</v>
       </c>
       <c r="M27" t="n">
-        <v>43.61323379359452</v>
+        <v>39.78256476579234</v>
       </c>
       <c r="N27" t="n">
         <v>0.3170479884975216</v>
@@ -2334,7 +2334,7 @@
         <v>0.053911791108084</v>
       </c>
       <c r="P27" t="n">
-        <v>137.5603548228645</v>
+        <v>125.4780544557952</v>
       </c>
       <c r="Q27" t="n">
         <v>205.9844559585492</v>
@@ -2372,13 +2372,13 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.4763480392156863</v>
+        <v>0.5</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4844559585492228</v>
+        <v>0.5</v>
       </c>
       <c r="H28" t="n">
-        <v>0.4361323379359452</v>
+        <v>0.3978256476579234</v>
       </c>
       <c r="I28" t="n">
         <v>386</v>
@@ -2389,13 +2389,13 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>47.63480392156863</v>
+        <v>50</v>
       </c>
       <c r="L28" t="n">
-        <v>48.44559585492228</v>
+        <v>50</v>
       </c>
       <c r="M28" t="n">
-        <v>43.61323379359452</v>
+        <v>39.78256476579234</v>
       </c>
       <c r="N28" t="n">
         <v>0.3170479884975216</v>
@@ -2404,7 +2404,7 @@
         <v>0.053911791108084</v>
       </c>
       <c r="P28" t="n">
-        <v>137.5603548228645</v>
+        <v>125.4780544557952</v>
       </c>
       <c r="Q28" t="n">
         <v>205.9844559585492</v>
@@ -2652,13 +2652,13 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.4733499033416183</v>
+        <v>0.4702048097704895</v>
       </c>
       <c r="G32" t="n">
-        <v>0.4792746113989637</v>
+        <v>0.4766839378238341</v>
       </c>
       <c r="H32" t="n">
-        <v>0.448630209998934</v>
+        <v>0.4465989098342039</v>
       </c>
       <c r="I32" t="n">
         <v>386</v>
@@ -2669,13 +2669,13 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>47.33499033416183</v>
+        <v>47.02048097704895</v>
       </c>
       <c r="L32" t="n">
-        <v>47.92746113989637</v>
+        <v>47.66839378238341</v>
       </c>
       <c r="M32" t="n">
-        <v>44.8630209998934</v>
+        <v>44.65989098342039</v>
       </c>
       <c r="N32" t="n">
         <v>1.890200869433597</v>
@@ -2684,7 +2684,7 @@
         <v>0.321415426441097</v>
       </c>
       <c r="P32" t="n">
-        <v>23.73452563977326</v>
+        <v>23.62706086195105</v>
       </c>
       <c r="Q32" t="n">
         <v>1288.764248704663</v>
@@ -2722,13 +2722,13 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.4733499033416183</v>
+        <v>0.4702048097704895</v>
       </c>
       <c r="G33" t="n">
-        <v>0.4792746113989637</v>
+        <v>0.4766839378238341</v>
       </c>
       <c r="H33" t="n">
-        <v>0.448630209998934</v>
+        <v>0.4465989098342039</v>
       </c>
       <c r="I33" t="n">
         <v>386</v>
@@ -2739,13 +2739,13 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>47.33499033416183</v>
+        <v>47.02048097704895</v>
       </c>
       <c r="L33" t="n">
-        <v>47.92746113989637</v>
+        <v>47.66839378238341</v>
       </c>
       <c r="M33" t="n">
-        <v>44.8630209998934</v>
+        <v>44.65989098342039</v>
       </c>
       <c r="N33" t="n">
         <v>1.890200869433597</v>
@@ -2754,7 +2754,7 @@
         <v>0.321415426441097</v>
       </c>
       <c r="P33" t="n">
-        <v>23.73452563977326</v>
+        <v>23.62706086195105</v>
       </c>
       <c r="Q33" t="n">
         <v>1288.764248704663</v>
@@ -2792,13 +2792,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0.4733499033416183</v>
+        <v>0.4702048097704895</v>
       </c>
       <c r="G34" t="n">
-        <v>0.4792746113989637</v>
+        <v>0.4766839378238341</v>
       </c>
       <c r="H34" t="n">
-        <v>0.448630209998934</v>
+        <v>0.4465989098342039</v>
       </c>
       <c r="I34" t="n">
         <v>386</v>
@@ -2809,13 +2809,13 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>47.33499033416183</v>
+        <v>47.02048097704895</v>
       </c>
       <c r="L34" t="n">
-        <v>47.92746113989637</v>
+        <v>47.66839378238341</v>
       </c>
       <c r="M34" t="n">
-        <v>44.8630209998934</v>
+        <v>44.65989098342039</v>
       </c>
       <c r="N34" t="n">
         <v>1.890200869433597</v>
@@ -2824,7 +2824,7 @@
         <v>0.321415426441097</v>
       </c>
       <c r="P34" t="n">
-        <v>23.73452563977326</v>
+        <v>23.62706086195105</v>
       </c>
       <c r="Q34" t="n">
         <v>1288.764248704663</v>
@@ -3072,13 +3072,13 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0.5313265456691751</v>
+        <v>0.5215305667112896</v>
       </c>
       <c r="G38" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.5103626943005182</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5176060206548011</v>
+        <v>0.437408906882591</v>
       </c>
       <c r="I38" t="n">
         <v>386</v>
@@ -3089,13 +3089,13 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>53.13265456691752</v>
+        <v>52.15305667112896</v>
       </c>
       <c r="L38" t="n">
-        <v>52.84974093264248</v>
+        <v>51.03626943005182</v>
       </c>
       <c r="M38" t="n">
-        <v>51.76060206548011</v>
+        <v>43.7408906882591</v>
       </c>
       <c r="N38" t="n">
         <v>0.5986731427653721</v>
@@ -3104,7 +3104,7 @@
         <v>0.1018001772152521</v>
       </c>
       <c r="P38" t="n">
-        <v>86.45886773271499</v>
+        <v>73.06305822608404</v>
       </c>
       <c r="Q38" t="n">
         <v>479.5466321243524</v>
@@ -3142,13 +3142,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.5313265456691751</v>
+        <v>0.5215305667112896</v>
       </c>
       <c r="G39" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.5103626943005182</v>
       </c>
       <c r="H39" t="n">
-        <v>0.5176060206548011</v>
+        <v>0.437408906882591</v>
       </c>
       <c r="I39" t="n">
         <v>386</v>
@@ -3159,13 +3159,13 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>53.13265456691752</v>
+        <v>52.15305667112896</v>
       </c>
       <c r="L39" t="n">
-        <v>52.84974093264248</v>
+        <v>51.03626943005182</v>
       </c>
       <c r="M39" t="n">
-        <v>51.76060206548011</v>
+        <v>43.7408906882591</v>
       </c>
       <c r="N39" t="n">
         <v>0.5986731427653721</v>
@@ -3174,7 +3174,7 @@
         <v>0.1018001772152521</v>
       </c>
       <c r="P39" t="n">
-        <v>86.45886773271499</v>
+        <v>73.06305822608404</v>
       </c>
       <c r="Q39" t="n">
         <v>479.5466321243524</v>
@@ -3212,13 +3212,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0.5313265456691751</v>
+        <v>0.5215305667112896</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5284974093264249</v>
+        <v>0.5103626943005182</v>
       </c>
       <c r="H40" t="n">
-        <v>0.5176060206548011</v>
+        <v>0.437408906882591</v>
       </c>
       <c r="I40" t="n">
         <v>386</v>
@@ -3229,13 +3229,13 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>53.13265456691752</v>
+        <v>52.15305667112896</v>
       </c>
       <c r="L40" t="n">
-        <v>52.84974093264248</v>
+        <v>51.03626943005182</v>
       </c>
       <c r="M40" t="n">
-        <v>51.76060206548011</v>
+        <v>43.7408906882591</v>
       </c>
       <c r="N40" t="n">
         <v>0.5986731427653721</v>
@@ -3244,7 +3244,7 @@
         <v>0.1018001772152521</v>
       </c>
       <c r="P40" t="n">
-        <v>86.45886773271499</v>
+        <v>73.06305822608404</v>
       </c>
       <c r="Q40" t="n">
         <v>479.5466321243524</v>
@@ -3928,13 +3928,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>49.9819791670712</v>
+        <v>50.83300466146378</v>
       </c>
       <c r="C2" t="n">
-        <v>50.09715025906736</v>
+        <v>50.29145077720207</v>
       </c>
       <c r="D2" t="n">
-        <v>47.87428456441207</v>
+        <v>44.5092997035469</v>
       </c>
     </row>
     <row r="3">
@@ -3996,13 +3996,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>51.62387544151312</v>
+        <v>52.97919755040581</v>
       </c>
       <c r="C2" t="n">
-        <v>51.44247865871895</v>
+        <v>51.73392943592102</v>
       </c>
       <c r="D2" t="n">
-        <v>49.60126812117924</v>
+        <v>47.97889860078693</v>
       </c>
     </row>
     <row r="3">
@@ -4012,13 +4012,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44.83500719256355</v>
+        <v>44.33071057806345</v>
       </c>
       <c r="C3" t="n">
-        <v>49.6492764373472</v>
+        <v>49.55212617827984</v>
       </c>
       <c r="D3" t="n">
-        <v>42.03845362561879</v>
+        <v>40.29583828514593</v>
       </c>
     </row>
   </sheetData>
@@ -4064,13 +4064,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>47.82746657113396</v>
+        <v>47.96135267432521</v>
       </c>
       <c r="C2" t="n">
-        <v>50.79422147548767</v>
+        <v>50.72945463610943</v>
       </c>
       <c r="D2" t="n">
-        <v>46.4688345518513</v>
+        <v>44.96214574916428</v>
       </c>
     </row>
     <row r="3">
@@ -4080,13 +4080,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.63141606294271</v>
+        <v>49.34855545414405</v>
       </c>
       <c r="C3" t="n">
-        <v>50.29753362057847</v>
+        <v>50.55660097809143</v>
       </c>
       <c r="D3" t="n">
-        <v>45.17088719494672</v>
+        <v>43.31259113676858</v>
       </c>
     </row>
   </sheetData>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45.77085008665296</v>
+        <v>46.66118925068466</v>
       </c>
       <c r="C2" t="n">
-        <v>50.44285450849165</v>
+        <v>50.66953844631549</v>
       </c>
       <c r="D2" t="n">
-        <v>43.846343848945</v>
+        <v>40.50675024013895</v>
       </c>
     </row>
     <row r="3">
@@ -4148,13 +4148,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50.68803254742372</v>
+        <v>50.6487188777846</v>
       </c>
       <c r="C3" t="n">
-        <v>50.64890058757448</v>
+        <v>50.61651716788537</v>
       </c>
       <c r="D3" t="n">
-        <v>47.79337789785303</v>
+        <v>47.7679866457939</v>
       </c>
     </row>
   </sheetData>

</xml_diff>